<commit_message>
result LKB vs MU
</commit_message>
<xml_diff>
--- a/javier_analysis/Krill_data/LKB_MUs.xlsx
+++ b/javier_analysis/Krill_data/LKB_MUs.xlsx
@@ -1,52 +1,62 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr date1904="false"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/86bd8becdb44c660/R-Git projects/WattKrug/javier_analysis/Krill_data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_C759D452AC861357A7819844360310B9A226F2E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A891C519-D0AB-438F-9EFA-721A40FDACAA}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="10">
   <si>
-    <t xml:space="preserve">cal.yr</t>
+    <t>cal.yr</t>
   </si>
   <si>
-    <t xml:space="preserve">season</t>
+    <t>season</t>
   </si>
   <si>
-    <t xml:space="preserve">density</t>
+    <t>density</t>
   </si>
   <si>
-    <t xml:space="preserve">MU</t>
+    <t>MU</t>
   </si>
   <si>
-    <t xml:space="preserve">biomass</t>
+    <t>biomass</t>
   </si>
   <si>
-    <t xml:space="preserve">S</t>
+    <t>S</t>
   </si>
   <si>
-    <t xml:space="preserve">BS</t>
+    <t>BS</t>
   </si>
   <si>
-    <t xml:space="preserve">W</t>
+    <t>W</t>
   </si>
   <si>
-    <t xml:space="preserve">SSIW</t>
+    <t>SSIW</t>
+  </si>
+  <si>
+    <t>catch</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -82,18 +92,27 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:E46" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:E46"/>
-  <tableColumns count="5">
-    <tableColumn id="1" name="cal.yr"/>
-    <tableColumn id="2" name="season"/>
-    <tableColumn id="3" name="density"/>
-    <tableColumn id="4" name="MU"/>
-    <tableColumn id="5" name="biomass"/>
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table3" displayName="Table3" ref="A1:F46" totalsRowShown="0">
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="cal.yr"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="season"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="density"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="MU"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="biomass"/>
+    <tableColumn id="6" xr3:uid="{95ED9246-D406-443E-B195-5C4A729ACE8D}" name="catch"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -377,11 +396,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F46"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -397,777 +416,780 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
+      <c r="F1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2">
         <v>1996</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2">
         <v>125.7325419</v>
       </c>
       <c r="D2" t="s">
         <v>6</v>
       </c>
-      <c r="E2" t="n">
-        <v>4426791.3352152</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
+      <c r="E2">
+        <v>4426791.3352151997</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
         <v>1997</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" t="n">
-        <v>33.31412531</v>
+      <c r="C3">
+        <v>33.314125310000001</v>
       </c>
       <c r="D3" t="s">
         <v>6</v>
       </c>
-      <c r="E3" t="n">
-        <v>1172923.72391448</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
+      <c r="E3">
+        <v>1172923.7239144801</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
         <v>1998</v>
       </c>
       <c r="B4" t="s">
         <v>5</v>
       </c>
-      <c r="C4" t="n">
-        <v>56.41132042</v>
+      <c r="C4">
+        <v>56.411320420000003</v>
       </c>
       <c r="D4" t="s">
         <v>6</v>
       </c>
-      <c r="E4" t="n">
-        <v>1986129.76934736</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
+      <c r="E4">
+        <v>1986129.7693473599</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
         <v>1999</v>
       </c>
       <c r="B5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5">
         <v>17.25651998</v>
       </c>
       <c r="D5" t="s">
         <v>6</v>
       </c>
-      <c r="E5" t="n">
-        <v>607567.55545584</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
+      <c r="E5">
+        <v>607567.55545583996</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6">
         <v>2000</v>
       </c>
       <c r="B6" t="s">
         <v>5</v>
       </c>
-      <c r="C6" t="n">
-        <v>70.91101198</v>
+      <c r="C6">
+        <v>70.911011979999998</v>
       </c>
       <c r="D6" t="s">
         <v>6</v>
       </c>
-      <c r="E6" t="n">
-        <v>2496634.90979184</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
+      <c r="E6">
+        <v>2496634.9097918398</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7">
         <v>2001</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7">
         <v>17.6515644405</v>
       </c>
       <c r="D7" t="s">
         <v>6</v>
       </c>
-      <c r="E7" t="n">
-        <v>621476.280821124</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
+      <c r="E7">
+        <v>621476.28082112398</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8">
         <v>2002</v>
       </c>
       <c r="B8" t="s">
         <v>5</v>
       </c>
-      <c r="C8" t="n">
-        <v>4.6986579325</v>
+      <c r="C8">
+        <v>4.6986579324999997</v>
       </c>
       <c r="D8" t="s">
         <v>6</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8">
         <v>165430.34848746</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="n">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9">
         <v>2003</v>
       </c>
       <c r="B9" t="s">
         <v>5</v>
       </c>
-      <c r="C9" t="n">
-        <v>48.475030395</v>
+      <c r="C9">
+        <v>48.475030394999997</v>
       </c>
       <c r="D9" t="s">
         <v>6</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9">
         <v>1706708.87014716</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="n">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10">
         <v>2004</v>
       </c>
       <c r="B10" t="s">
         <v>5</v>
       </c>
-      <c r="C10" t="n">
-        <v>1.7472106385</v>
+      <c r="C10">
+        <v>1.7472106384999999</v>
       </c>
       <c r="D10" t="s">
         <v>6</v>
       </c>
-      <c r="E10" t="n">
-        <v>61515.792160308</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
+      <c r="E10">
+        <v>61515.792160308003</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11">
         <v>2005</v>
       </c>
       <c r="B11" t="s">
         <v>5</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11">
         <v>13.2948315745</v>
       </c>
       <c r="D11" t="s">
         <v>6</v>
       </c>
-      <c r="E11" t="n">
-        <v>468084.430074996</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
+      <c r="E11">
+        <v>468084.43007499602</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12">
         <v>2006</v>
       </c>
       <c r="B12" t="s">
         <v>5</v>
       </c>
-      <c r="C12" t="n">
-        <v>35.64579129</v>
+      <c r="C12">
+        <v>35.645791289999998</v>
       </c>
       <c r="D12" t="s">
         <v>6</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12">
         <v>1255017.01973832</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="n">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13">
         <v>2007</v>
       </c>
       <c r="B13" t="s">
         <v>5</v>
       </c>
-      <c r="C13" t="n">
-        <v>56.58966285</v>
+      <c r="C13">
+        <v>56.589662850000003</v>
       </c>
       <c r="D13" t="s">
         <v>6</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13">
         <v>1992408.8496228</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="n">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14">
         <v>2008</v>
       </c>
       <c r="B14" t="s">
         <v>5</v>
       </c>
-      <c r="C14" t="n">
-        <v>94.831777175</v>
+      <c r="C14">
+        <v>94.831777174999999</v>
       </c>
       <c r="D14" t="s">
         <v>6</v>
       </c>
-      <c r="E14" t="n">
-        <v>3338837.2107774</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
+      <c r="E14">
+        <v>3338837.2107774001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15">
         <v>2009</v>
       </c>
       <c r="B15" t="s">
         <v>5</v>
       </c>
-      <c r="C15" t="n">
-        <v>28.72228523</v>
+      <c r="C15">
+        <v>28.722285230000001</v>
       </c>
       <c r="D15" t="s">
         <v>6</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15">
         <v>1011254.21837784</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="n">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16">
         <v>2010</v>
       </c>
       <c r="B16" t="s">
         <v>5</v>
       </c>
-      <c r="C16" t="n">
-        <v>9.109248864</v>
+      <c r="C16">
+        <v>9.1092488639999996</v>
       </c>
       <c r="D16" t="s">
         <v>6</v>
       </c>
-      <c r="E16" t="n">
-        <v>320718.434003712</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
+      <c r="E16">
+        <v>320718.43400371203</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17">
         <v>2011</v>
       </c>
       <c r="B17" t="s">
         <v>5</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C17">
         <v>41.75105722</v>
       </c>
       <c r="D17" t="s">
         <v>6</v>
       </c>
-      <c r="E17" t="n">
-        <v>1469971.22260176</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
+      <c r="E17">
+        <v>1469971.2226017599</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18">
         <v>2014</v>
       </c>
       <c r="B18" t="s">
         <v>7</v>
       </c>
-      <c r="C18" t="n">
+      <c r="C18">
         <v>130.9908417</v>
       </c>
       <c r="D18" t="s">
         <v>6</v>
       </c>
-      <c r="E18" t="n">
-        <v>4611925.5545736</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
+      <c r="E18">
+        <v>4611925.5545736002</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19">
         <v>2015</v>
       </c>
       <c r="B19" t="s">
         <v>7</v>
       </c>
-      <c r="C19" t="n">
-        <v>3.639688383</v>
+      <c r="C19">
+        <v>3.6396883830000002</v>
       </c>
       <c r="D19" t="s">
         <v>6</v>
       </c>
-      <c r="E19" t="n">
+      <c r="E19">
         <v>128146.148588664</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="n">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20">
         <v>1996</v>
       </c>
       <c r="B20" t="s">
         <v>5</v>
       </c>
-      <c r="C20" t="n">
+      <c r="C20">
         <v>108.13134578</v>
       </c>
       <c r="D20" t="s">
         <v>8</v>
       </c>
-      <c r="E20" t="n">
-        <v>5096662.85199452</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
+      <c r="E20">
+        <v>5096662.8519945201</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21">
         <v>1997</v>
       </c>
       <c r="B21" t="s">
         <v>5</v>
       </c>
-      <c r="C21" t="n">
-        <v>210.3628151</v>
+      <c r="C21">
+        <v>210.36281510000001</v>
       </c>
       <c r="D21" t="s">
         <v>8</v>
       </c>
-      <c r="E21" t="n">
-        <v>9915240.9269234</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
+      <c r="E21">
+        <v>9915240.9269233998</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22">
         <v>1998</v>
       </c>
       <c r="B22" t="s">
         <v>5</v>
       </c>
-      <c r="C22" t="n">
-        <v>92.75483719</v>
+      <c r="C22">
+        <v>92.754837190000003</v>
       </c>
       <c r="D22" t="s">
         <v>8</v>
       </c>
-      <c r="E22" t="n">
-        <v>4371906.49611346</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
+      <c r="E22">
+        <v>4371906.4961134596</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23">
         <v>1999</v>
       </c>
       <c r="B23" t="s">
         <v>5</v>
       </c>
-      <c r="C23" t="n">
-        <v>38.92547241</v>
+      <c r="C23">
+        <v>38.925472409999998</v>
       </c>
       <c r="D23" t="s">
         <v>8</v>
       </c>
-      <c r="E23" t="n">
-        <v>1834713.21657294</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
+      <c r="E23">
+        <v>1834713.2165729399</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24">
         <v>2000</v>
       </c>
       <c r="B24" t="s">
         <v>5</v>
       </c>
-      <c r="C24" t="n">
+      <c r="C24">
         <v>119.273724</v>
       </c>
       <c r="D24" t="s">
         <v>8</v>
       </c>
-      <c r="E24" t="n">
-        <v>5621847.707016</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
+      <c r="E24">
+        <v>5621847.7070159996</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25">
         <v>2001</v>
       </c>
       <c r="B25" t="s">
         <v>5</v>
       </c>
-      <c r="C25" t="n">
+      <c r="C25">
         <v>30.58777491</v>
       </c>
       <c r="D25" t="s">
         <v>8</v>
       </c>
-      <c r="E25" t="n">
-        <v>1441724.18260794</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
+      <c r="E25">
+        <v>1441724.1826079399</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26">
         <v>2002</v>
       </c>
       <c r="B26" t="s">
         <v>5</v>
       </c>
-      <c r="C26" t="n">
+      <c r="C26">
         <v>14.42591258</v>
       </c>
       <c r="D26" t="s">
         <v>8</v>
       </c>
-      <c r="E26" t="n">
-        <v>679950.96354572</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
+      <c r="E26">
+        <v>679950.96354571998</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27">
         <v>2003</v>
       </c>
       <c r="B27" t="s">
         <v>5</v>
       </c>
-      <c r="C27" t="n">
-        <v>68.5010684</v>
+      <c r="C27">
+        <v>68.501068399999994</v>
       </c>
       <c r="D27" t="s">
         <v>8</v>
       </c>
-      <c r="E27" t="n">
-        <v>3228729.3579656</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
+      <c r="E27">
+        <v>3228729.3579656002</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28">
         <v>2004</v>
       </c>
       <c r="B28" t="s">
         <v>5</v>
       </c>
-      <c r="C28" t="n">
-        <v>16.27905747</v>
+      <c r="C28">
+        <v>16.279057470000001</v>
       </c>
       <c r="D28" t="s">
         <v>8</v>
       </c>
-      <c r="E28" t="n">
-        <v>767297.09479098</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
+      <c r="E28">
+        <v>767297.09479097999</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29">
         <v>2005</v>
       </c>
       <c r="B29" t="s">
         <v>5</v>
       </c>
-      <c r="C29" t="n">
+      <c r="C29">
         <v>46.365782775</v>
       </c>
       <c r="D29" t="s">
         <v>8</v>
       </c>
-      <c r="E29" t="n">
-        <v>2185404.80531685</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
+      <c r="E29">
+        <v>2185404.8053168501</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30">
         <v>2006</v>
       </c>
       <c r="B30" t="s">
         <v>5</v>
       </c>
-      <c r="C30" t="n">
-        <v>61.74483825</v>
+      <c r="C30">
+        <v>61.744838250000001</v>
       </c>
       <c r="D30" t="s">
         <v>8</v>
       </c>
-      <c r="E30" t="n">
-        <v>2910281.2060755</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
+      <c r="E30">
+        <v>2910281.2060755002</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31">
         <v>2007</v>
       </c>
       <c r="B31" t="s">
         <v>5</v>
       </c>
-      <c r="C31" t="n">
+      <c r="C31">
         <v>132.8970367</v>
       </c>
       <c r="D31" t="s">
         <v>8</v>
       </c>
-      <c r="E31" t="n">
-        <v>6263968.9278178</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
+      <c r="E31">
+        <v>6263968.9278178001</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32">
         <v>2008</v>
       </c>
       <c r="B32" t="s">
         <v>5</v>
       </c>
-      <c r="C32" t="n">
-        <v>133.5747287</v>
+      <c r="C32">
+        <v>133.57472870000001</v>
       </c>
       <c r="D32" t="s">
         <v>8</v>
       </c>
-      <c r="E32" t="n">
-        <v>6295911.2625458</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
+      <c r="E32">
+        <v>6295911.2625457998</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33">
         <v>2009</v>
       </c>
       <c r="B33" t="s">
         <v>5</v>
       </c>
-      <c r="C33" t="n">
+      <c r="C33">
         <v>112.125612</v>
       </c>
       <c r="D33" t="s">
         <v>8</v>
       </c>
-      <c r="E33" t="n">
+      <c r="E33">
         <v>5284928.596008</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="n">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34">
         <v>2010</v>
       </c>
       <c r="B34" t="s">
         <v>5</v>
       </c>
-      <c r="C34" t="n">
-        <v>24.1142837</v>
+      <c r="C34">
+        <v>24.114283700000001</v>
       </c>
       <c r="D34" t="s">
         <v>8</v>
       </c>
-      <c r="E34" t="n">
-        <v>1136602.6479158</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
+      <c r="E34">
+        <v>1136602.6479158001</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35">
         <v>2011</v>
       </c>
       <c r="B35" t="s">
         <v>5</v>
       </c>
-      <c r="C35" t="n">
+      <c r="C35">
         <v>106.4585503</v>
       </c>
       <c r="D35" t="s">
         <v>8</v>
       </c>
-      <c r="E35" t="n">
-        <v>5017817.3098402</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
+      <c r="E35">
+        <v>5017817.3098401995</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36">
         <v>2014</v>
       </c>
       <c r="B36" t="s">
         <v>7</v>
       </c>
-      <c r="C36" t="n">
-        <v>4.652919263</v>
+      <c r="C36">
+        <v>4.6529192630000002</v>
       </c>
       <c r="D36" t="s">
         <v>8</v>
       </c>
-      <c r="E36" t="n">
-        <v>219310.696542242</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
+      <c r="E36">
+        <v>219310.69654224199</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37">
         <v>2013</v>
       </c>
       <c r="B37" t="s">
         <v>5</v>
       </c>
-      <c r="C37" t="n">
+      <c r="C37">
         <v>18</v>
       </c>
       <c r="D37" t="s">
         <v>8</v>
       </c>
-      <c r="E37" t="n">
+      <c r="E37">
         <v>848412</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="n">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38">
         <v>2015</v>
       </c>
       <c r="B38" t="s">
         <v>5</v>
       </c>
-      <c r="C38" t="n">
-        <v>19.6</v>
+      <c r="C38">
+        <v>19.600000000000001</v>
       </c>
       <c r="D38" t="s">
         <v>8</v>
       </c>
-      <c r="E38" t="n">
+      <c r="E38">
         <v>923826.4</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="n">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39">
         <v>2016</v>
       </c>
       <c r="B39" t="s">
         <v>5</v>
       </c>
-      <c r="C39" t="n">
+      <c r="C39">
         <v>38.5</v>
       </c>
       <c r="D39" t="s">
         <v>8</v>
       </c>
-      <c r="E39" t="n">
+      <c r="E39">
         <v>1814659</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="n">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40">
         <v>2018</v>
       </c>
       <c r="B40" t="s">
         <v>5</v>
       </c>
-      <c r="C40" t="n">
+      <c r="C40">
         <v>77</v>
       </c>
       <c r="D40" t="s">
         <v>8</v>
       </c>
-      <c r="E40" t="n">
+      <c r="E40">
         <v>3629318</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="n">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41">
         <v>2019</v>
       </c>
       <c r="B41" t="s">
         <v>5</v>
       </c>
-      <c r="C41" t="n">
+      <c r="C41">
         <v>62.9</v>
       </c>
       <c r="D41" t="s">
         <v>8</v>
       </c>
-      <c r="E41" t="n">
+      <c r="E41">
         <v>2964728.6</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="n">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42">
         <v>2013</v>
       </c>
       <c r="B42" t="s">
         <v>5</v>
       </c>
-      <c r="C42" t="n">
+      <c r="C42">
         <v>25.1</v>
       </c>
       <c r="D42" t="s">
         <v>6</v>
       </c>
-      <c r="E42" t="n">
+      <c r="E42">
         <v>883720.8</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="n">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43">
         <v>2015</v>
       </c>
       <c r="B43" t="s">
         <v>5</v>
       </c>
-      <c r="C43" t="n">
-        <v>17.6</v>
+      <c r="C43">
+        <v>17.600000000000001</v>
       </c>
       <c r="D43" t="s">
         <v>6</v>
       </c>
-      <c r="E43" t="n">
-        <v>619660.8</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
+      <c r="E43">
+        <v>619660.80000000005</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44">
         <v>2016</v>
       </c>
       <c r="B44" t="s">
         <v>5</v>
       </c>
-      <c r="C44" t="n">
+      <c r="C44">
         <v>46.2</v>
       </c>
       <c r="D44" t="s">
         <v>6</v>
       </c>
-      <c r="E44" t="n">
+      <c r="E44">
         <v>1626609.6</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="n">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45">
         <v>2018</v>
       </c>
       <c r="B45" t="s">
         <v>5</v>
       </c>
-      <c r="C45" t="n">
+      <c r="C45">
         <v>35.6</v>
       </c>
       <c r="D45" t="s">
         <v>6</v>
       </c>
-      <c r="E45" t="n">
+      <c r="E45">
         <v>1253404.8</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="n">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46">
         <v>2019</v>
       </c>
       <c r="B46" t="s">
         <v>5</v>
       </c>
-      <c r="C46" t="n">
+      <c r="C46">
         <v>77.2</v>
       </c>
       <c r="D46" t="s">
         <v>6</v>
       </c>
-      <c r="E46" t="n">
+      <c r="E46">
         <v>2718057.6</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>